<commit_message>
Update listings: 2026-07-07 14:37 UTC
</commit_message>
<xml_diff>
--- a/listings.xlsx
+++ b/listings.xlsx
@@ -53,24 +53,30 @@
     <t>PARIS 7ÈME</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>https://www.barnes-international.com/en/for-rent/france/paris-7eme/ref-APM-87108484.html</t>
+  </si>
+  <si>
+    <t>PARIS 16ÈME</t>
+  </si>
+  <si>
+    <t>https://www.barnes-international.com/en/for-rent/france/paris-16eme/ref-APM-87141456.html</t>
+  </si>
+  <si>
+    <t>https://www.barnes-international.com/en/for-rent/france/paris-16eme/ref-APM-87146307.html</t>
+  </si>
+  <si>
+    <t>https://www.barnes-international.com/en/for-rent/france/paris-7eme/ref-APM-87135906.html</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>https://www.barnes-international.com/en/for-rent/france/paris-7eme/ref-APM-87108484.html</t>
-  </si>
-  <si>
-    <t>PARIS 16ÈME</t>
-  </si>
-  <si>
-    <t>https://www.barnes-international.com/en/for-rent/france/paris-16eme/ref-APM-87141456.html</t>
-  </si>
-  <si>
-    <t>https://www.barnes-international.com/en/for-rent/france/paris-16eme/ref-APM-87146307.html</t>
-  </si>
-  <si>
-    <t>https://www.barnes-international.com/en/for-rent/france/paris-7eme/ref-APM-87135906.html</t>
-  </si>
-  <si>
     <t>https://www.barnes-international.com/en/for-rent/france/paris-7eme/ref-APM-87108483.html</t>
   </si>
   <si>
@@ -410,12 +416,6 @@
     <t>Paris 15ème</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/273206899.htm</t>
   </si>
   <si>
@@ -452,10 +452,10 @@
     <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/273639859.htm</t>
   </si>
   <si>
-    <t>1 / 14</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/boulogne-billancourt-92/274285499.htm</t>
+    <t>1 / 15</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/montreuil-93/ruffins-theophile-sueur-montreau-le-morillon/270926483.htm</t>
   </si>
   <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/273639863.htm</t>
@@ -512,10 +512,10 @@
     <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/cambronne-garibaldi/274316193.htm</t>
   </si>
   <si>
-    <t>Nouveau</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/saint-ouen-93/marie-godillot-landy/273787275.htm</t>
+    <t>1 941 € /mois</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/issy-les-moulineaux-92/273103027.htm</t>
   </si>
   <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273630989.htm</t>
@@ -548,7 +548,7 @@
     <t>Prospector — Paris Listings</t>
   </si>
   <si>
-    <t>Generated: 07/07/2026, 14:13:39</t>
+    <t>Generated: 07/07/2026, 14:37:55</t>
   </si>
   <si>
     <t>Barnes: 100 listings</t>
@@ -1042,13 +1042,13 @@
         <v>13</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1071,7 +1071,7 @@
         <f>B3/E3</f>
       </c>
       <c r="G3" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>13</v>
@@ -1083,7 +1083,7 @@
         <v>13</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1106,19 +1106,19 @@
         <f>B4/E4</f>
       </c>
       <c r="G4" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1147,13 +1147,13 @@
         <v>13</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1179,16 +1179,16 @@
         <v>12</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1211,19 +1211,19 @@
         <f>B7/E7</f>
       </c>
       <c r="G7" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1246,7 +1246,7 @@
         <f>B8/E8</f>
       </c>
       <c r="G8" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>13</v>
@@ -1258,7 +1258,7 @@
         <v>13</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1281,7 +1281,7 @@
         <f>B9/E9</f>
       </c>
       <c r="G9" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>13</v>
@@ -1290,10 +1290,10 @@
         <v>13</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1322,13 +1322,13 @@
         <v>13</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1349,19 +1349,19 @@
         <f>B11/E11</f>
       </c>
       <c r="G11" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1382,19 +1382,19 @@
         <f>B12/E12</f>
       </c>
       <c r="G12" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1417,19 +1417,19 @@
         <f>B13/E13</f>
       </c>
       <c r="G13" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1452,19 +1452,19 @@
         <f>B14/E14</f>
       </c>
       <c r="G14" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1487,7 +1487,7 @@
         <f>B15/E15</f>
       </c>
       <c r="G15" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>13</v>
@@ -1499,7 +1499,7 @@
         <v>13</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1518,19 +1518,19 @@
         <f>B16/E16</f>
       </c>
       <c r="G16" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1553,19 +1553,19 @@
         <f>B17/E17</f>
       </c>
       <c r="G17" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1588,19 +1588,19 @@
         <f>B18/E18</f>
       </c>
       <c r="G18" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1619,19 +1619,19 @@
         <f>B19/E19</f>
       </c>
       <c r="G19" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1654,19 +1654,19 @@
         <f>B20/E20</f>
       </c>
       <c r="G20" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1689,19 +1689,19 @@
         <f>B21/E21</f>
       </c>
       <c r="G21" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1724,19 +1724,19 @@
         <f>B22/E22</f>
       </c>
       <c r="G22" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1759,19 +1759,19 @@
         <f>B23/E23</f>
       </c>
       <c r="G23" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1794,19 +1794,19 @@
         <f>B24/E24</f>
       </c>
       <c r="G24" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1829,19 +1829,19 @@
         <f>B25/E25</f>
       </c>
       <c r="G25" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1864,19 +1864,19 @@
         <f>B26/E26</f>
       </c>
       <c r="G26" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1899,19 +1899,19 @@
         <f>B27/E27</f>
       </c>
       <c r="G27" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1934,7 +1934,7 @@
         <f>B28/E28</f>
       </c>
       <c r="G28" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>13</v>
@@ -1946,7 +1946,7 @@
         <v>13</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1975,13 +1975,13 @@
         <v>13</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2004,7 +2004,7 @@
         <f>B30/E30</f>
       </c>
       <c r="G30" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>13</v>
@@ -2013,10 +2013,10 @@
         <v>13</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2039,7 +2039,7 @@
         <f>B31/E31</f>
       </c>
       <c r="G31" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>13</v>
@@ -2051,7 +2051,7 @@
         <v>13</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2083,10 +2083,10 @@
         <v>13</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2112,16 +2112,16 @@
         <v>12</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2144,19 +2144,19 @@
         <f>B34/E34</f>
       </c>
       <c r="G34" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2177,19 +2177,19 @@
         <f>B35/E35</f>
       </c>
       <c r="G35" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2212,19 +2212,19 @@
         <f>B36/E36</f>
       </c>
       <c r="G36" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2250,16 +2250,16 @@
         <v>12</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J37" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="38" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2291,10 +2291,10 @@
         <v>13</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2317,19 +2317,19 @@
         <f>B39/E39</f>
       </c>
       <c r="G39" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J39" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2358,13 +2358,13 @@
         <v>13</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J40" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2387,19 +2387,19 @@
         <f>B41/E41</f>
       </c>
       <c r="G41" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2428,13 +2428,13 @@
         <v>13</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J42" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2469,7 +2469,7 @@
         <v>13</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2498,13 +2498,13 @@
         <v>13</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="45" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2527,19 +2527,19 @@
         <f>B45/E45</f>
       </c>
       <c r="G45" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J45" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2562,19 +2562,19 @@
         <f>B46/E46</f>
       </c>
       <c r="G46" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J46" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K46" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2597,19 +2597,19 @@
         <f>B47/E47</f>
       </c>
       <c r="G47" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H47" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2632,7 +2632,7 @@
         <f>B48/E48</f>
       </c>
       <c r="G48" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H48" s="3" t="s">
         <v>13</v>
@@ -2644,7 +2644,7 @@
         <v>13</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2676,10 +2676,10 @@
         <v>13</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K49" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="50" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2702,19 +2702,19 @@
         <f>B50/E50</f>
       </c>
       <c r="G50" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="51" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2737,7 +2737,7 @@
         <f>B51/E51</f>
       </c>
       <c r="G51" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>13</v>
@@ -2749,7 +2749,7 @@
         <v>13</v>
       </c>
       <c r="K51" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2772,7 +2772,7 @@
         <f>B52/E52</f>
       </c>
       <c r="G52" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>13</v>
@@ -2784,7 +2784,7 @@
         <v>13</v>
       </c>
       <c r="K52" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="53" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2807,7 +2807,7 @@
         <f>B53/E53</f>
       </c>
       <c r="G53" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>13</v>
@@ -2816,10 +2816,10 @@
         <v>13</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K53" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="54" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2842,19 +2842,19 @@
         <f>B54/E54</f>
       </c>
       <c r="G54" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J54" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K54" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="55" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2877,19 +2877,19 @@
         <f>B55/E55</f>
       </c>
       <c r="G55" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K55" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="56" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2912,7 +2912,7 @@
         <f>B56/E56</f>
       </c>
       <c r="G56" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>13</v>
@@ -2924,7 +2924,7 @@
         <v>13</v>
       </c>
       <c r="K56" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="57" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2947,19 +2947,19 @@
         <f>B57/E57</f>
       </c>
       <c r="G57" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H57" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J57" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="58" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2982,19 +2982,19 @@
         <f>B58/E58</f>
       </c>
       <c r="G58" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K58" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="59" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3017,19 +3017,19 @@
         <f>B59/E59</f>
       </c>
       <c r="G59" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H59" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J59" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K59" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="60" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3058,13 +3058,13 @@
         <v>13</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K60" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="61" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3099,7 +3099,7 @@
         <v>13</v>
       </c>
       <c r="K61" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="62" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3122,7 +3122,7 @@
         <f>B62/E62</f>
       </c>
       <c r="G62" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H62" s="3" t="s">
         <v>13</v>
@@ -3131,10 +3131,10 @@
         <v>13</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K62" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="63" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3157,19 +3157,19 @@
         <f>B63/E63</f>
       </c>
       <c r="G63" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H63" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J63" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K63" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="64" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3192,7 +3192,7 @@
         <f>B64/E64</f>
       </c>
       <c r="G64" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H64" s="3" t="s">
         <v>13</v>
@@ -3201,10 +3201,10 @@
         <v>13</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K64" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="65" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3227,19 +3227,19 @@
         <f>B65/E65</f>
       </c>
       <c r="G65" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J65" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K65" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="66" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3262,19 +3262,19 @@
         <f>B66/E66</f>
       </c>
       <c r="G66" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H66" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J66" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K66" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="67" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3300,16 +3300,16 @@
         <v>12</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J67" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K67" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="68" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3332,19 +3332,19 @@
         <f>B68/E68</f>
       </c>
       <c r="G68" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H68" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J68" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="69" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3367,19 +3367,19 @@
         <f>B69/E69</f>
       </c>
       <c r="G69" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H69" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J69" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K69" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="70" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3402,19 +3402,19 @@
         <f>B70/E70</f>
       </c>
       <c r="G70" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H70" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J70" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K70" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="71" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3437,7 +3437,7 @@
         <f>B71/E71</f>
       </c>
       <c r="G71" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H71" s="3" t="s">
         <v>13</v>
@@ -3449,7 +3449,7 @@
         <v>13</v>
       </c>
       <c r="K71" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="72" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3472,19 +3472,19 @@
         <f>B72/E72</f>
       </c>
       <c r="G72" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H72" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J72" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K72" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3507,7 +3507,7 @@
         <f>B73/E73</f>
       </c>
       <c r="G73" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H73" s="3" t="s">
         <v>13</v>
@@ -3516,10 +3516,10 @@
         <v>13</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K73" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="74" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3542,19 +3542,19 @@
         <f>B74/E74</f>
       </c>
       <c r="G74" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H74" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J74" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K74" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="75" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3577,7 +3577,7 @@
         <f>B75/E75</f>
       </c>
       <c r="G75" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>13</v>
@@ -3589,7 +3589,7 @@
         <v>13</v>
       </c>
       <c r="K75" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="76" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3612,19 +3612,19 @@
         <f>B76/E76</f>
       </c>
       <c r="G76" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J76" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K76" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="77" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3643,19 +3643,19 @@
         <f>B77/E77</f>
       </c>
       <c r="G77" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H77" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J77" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K77" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="78" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3684,13 +3684,13 @@
         <v>13</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J78" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K78" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="79" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3719,13 +3719,13 @@
         <v>13</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J79" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K79" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="80" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3748,19 +3748,19 @@
         <f>B80/E80</f>
       </c>
       <c r="G80" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H80" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J80" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K80" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="81" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3783,19 +3783,19 @@
         <f>B81/E81</f>
       </c>
       <c r="G81" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H81" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K81" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="82" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3818,7 +3818,7 @@
         <f>B82/E82</f>
       </c>
       <c r="G82" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H82" s="3" t="s">
         <v>13</v>
@@ -3830,7 +3830,7 @@
         <v>13</v>
       </c>
       <c r="K82" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="83" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3853,19 +3853,19 @@
         <f>B83/E83</f>
       </c>
       <c r="G83" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H83" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J83" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K83" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="84" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3900,7 +3900,7 @@
         <v>13</v>
       </c>
       <c r="K84" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="85" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3923,19 +3923,19 @@
         <f>B85/E85</f>
       </c>
       <c r="G85" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H85" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J85" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K85" s="3" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="86" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3958,19 +3958,19 @@
         <f>B86/E86</f>
       </c>
       <c r="G86" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J86" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K86" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="87" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3993,19 +3993,19 @@
         <f>B87/E87</f>
       </c>
       <c r="G87" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H87" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K87" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="88" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4028,7 +4028,7 @@
         <f>B88/E88</f>
       </c>
       <c r="G88" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H88" s="3" t="s">
         <v>13</v>
@@ -4037,10 +4037,10 @@
         <v>13</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K88" s="3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="89" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4063,7 +4063,7 @@
         <f>B89/E89</f>
       </c>
       <c r="G89" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H89" s="3" t="s">
         <v>13</v>
@@ -4075,7 +4075,7 @@
         <v>13</v>
       </c>
       <c r="K89" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="90" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4098,19 +4098,19 @@
         <f>B90/E90</f>
       </c>
       <c r="G90" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H90" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J90" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K90" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="91" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4133,7 +4133,7 @@
         <f>B91/E91</f>
       </c>
       <c r="G91" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H91" s="3" t="s">
         <v>13</v>
@@ -4145,7 +4145,7 @@
         <v>13</v>
       </c>
       <c r="K91" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="92" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4168,19 +4168,19 @@
         <f>B92/E92</f>
       </c>
       <c r="G92" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H92" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J92" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K92" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="93" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4203,19 +4203,19 @@
         <f>B93/E93</f>
       </c>
       <c r="G93" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H93" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J93" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K93" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="94" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4238,19 +4238,19 @@
         <f>B94/E94</f>
       </c>
       <c r="G94" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H94" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K94" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="95" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4273,7 +4273,7 @@
         <f>B95/E95</f>
       </c>
       <c r="G95" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H95" s="3" t="s">
         <v>13</v>
@@ -4285,7 +4285,7 @@
         <v>13</v>
       </c>
       <c r="K95" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="96" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4308,7 +4308,7 @@
         <f>B96/E96</f>
       </c>
       <c r="G96" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H96" s="3" t="s">
         <v>13</v>
@@ -4320,7 +4320,7 @@
         <v>13</v>
       </c>
       <c r="K96" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="97" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4343,19 +4343,19 @@
         <f>B97/E97</f>
       </c>
       <c r="G97" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H97" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J97" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K97" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="98" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4378,19 +4378,19 @@
         <f>B98/E98</f>
       </c>
       <c r="G98" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H98" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I98" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J98" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K98" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="99" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4419,13 +4419,13 @@
         <v>13</v>
       </c>
       <c r="I99" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K99" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="100" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4451,16 +4451,16 @@
         <v>12</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I100" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J100" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K100" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="101" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -4483,24 +4483,24 @@
         <f>B101/E101</f>
       </c>
       <c r="G101" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H101" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I101" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J101" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K101" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="102" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B102" s="4">
         <v>2200</v>
@@ -4518,16 +4518,16 @@
         <f>B102/E102</f>
       </c>
       <c r="G102" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I102" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J102" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K102" s="3" t="s">
         <v>134</v>
@@ -4535,7 +4535,7 @@
     </row>
     <row r="103" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B103" s="4">
         <v>7900</v>
@@ -4556,13 +4556,13 @@
         <v>135</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="I103" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J103" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K103" s="3" t="s">
         <v>136</v>
@@ -4570,7 +4570,7 @@
     </row>
     <row r="104" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B104" s="4">
         <v>6330</v>
@@ -4591,13 +4591,13 @@
         <v>137</v>
       </c>
       <c r="H104" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I104" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J104" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K104" s="3" t="s">
         <v>138</v>
@@ -4605,7 +4605,7 @@
     </row>
     <row r="105" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B105" s="4">
         <v>4700</v>
@@ -4623,16 +4623,16 @@
         <f>B105/E105</f>
       </c>
       <c r="G105" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I105" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J105" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K105" s="3" t="s">
         <v>139</v>
@@ -4640,7 +4640,7 @@
     </row>
     <row r="106" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B106" s="4">
         <v>2700</v>
@@ -4658,16 +4658,16 @@
         <f>B106/E106</f>
       </c>
       <c r="G106" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H106" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J106" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K106" s="3" t="s">
         <v>140</v>
@@ -4675,7 +4675,7 @@
     </row>
     <row r="107" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B107" s="4">
         <v>2250</v>
@@ -4693,16 +4693,16 @@
         <f>B107/E107</f>
       </c>
       <c r="G107" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H107" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="J107" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K107" s="3" t="s">
         <v>141</v>
@@ -4710,7 +4710,7 @@
     </row>
     <row r="108" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B108" s="4">
         <v>4150</v>
@@ -4731,13 +4731,13 @@
         <v>142</v>
       </c>
       <c r="H108" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I108" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J108" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K108" s="3" t="s">
         <v>143</v>
@@ -4745,7 +4745,7 @@
     </row>
     <row r="109" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B109" s="4">
         <v>1890</v>
@@ -4763,16 +4763,16 @@
         <f>B109/E109</f>
       </c>
       <c r="G109" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H109" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I109" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J109" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K109" s="3" t="s">
         <v>144</v>
@@ -4780,7 +4780,7 @@
     </row>
     <row r="110" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B110" s="4">
         <v>1100</v>
@@ -4801,13 +4801,13 @@
         <v>142</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J110" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K110" s="3" t="s">
         <v>145</v>
@@ -4815,19 +4815,19 @@
     </row>
     <row r="111" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B111" s="4">
-        <v>1350</v>
+        <v>1525</v>
       </c>
       <c r="C111" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D111" s="3">
         <v>1</v>
       </c>
       <c r="E111" s="3">
-        <v>46</v>
+        <v>66.1</v>
       </c>
       <c r="F111" s="5">
         <f>B111/E111</f>
@@ -4836,13 +4836,13 @@
         <v>146</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="I111" s="3" t="s">
-        <v>133</v>
+        <v>13</v>
       </c>
       <c r="J111" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K111" s="3" t="s">
         <v>147</v>
@@ -4850,7 +4850,7 @@
     </row>
     <row r="112" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B112" s="4">
         <v>1100</v>
@@ -4871,13 +4871,13 @@
         <v>142</v>
       </c>
       <c r="H112" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I112" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J112" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K112" s="3" t="s">
         <v>148</v>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="113" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B113" s="4">
         <v>2100</v>
@@ -4906,13 +4906,13 @@
         <v>149</v>
       </c>
       <c r="H113" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I113" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="J113" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K113" s="3" t="s">
         <v>150</v>
@@ -4920,7 +4920,7 @@
     </row>
     <row r="114" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B114" s="4">
         <v>1603</v>
@@ -4941,13 +4941,13 @@
         <v>151</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I114" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J114" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K114" s="3" t="s">
         <v>152</v>
@@ -4955,7 +4955,7 @@
     </row>
     <row r="115" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B115" s="4">
         <v>2200</v>
@@ -4976,13 +4976,13 @@
         <v>135</v>
       </c>
       <c r="H115" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I115" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J115" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K115" s="3" t="s">
         <v>153</v>
@@ -4990,7 +4990,7 @@
     </row>
     <row r="116" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B116" s="4">
         <v>162190</v>
@@ -5011,13 +5011,13 @@
         <v>154</v>
       </c>
       <c r="H116" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I116" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J116" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K116" s="3" t="s">
         <v>155</v>
@@ -5025,7 +5025,7 @@
     </row>
     <row r="117" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B117" s="4">
         <v>3650</v>
@@ -5046,13 +5046,13 @@
         <v>149</v>
       </c>
       <c r="H117" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I117" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="J117" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K117" s="3" t="s">
         <v>156</v>
@@ -5060,7 +5060,7 @@
     </row>
     <row r="118" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B118" s="4">
         <v>7250</v>
@@ -5081,13 +5081,13 @@
         <v>157</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="I118" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J118" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K118" s="3" t="s">
         <v>158</v>
@@ -5095,7 +5095,7 @@
     </row>
     <row r="119" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B119" s="4">
         <v>1500</v>
@@ -5116,13 +5116,13 @@
         <v>159</v>
       </c>
       <c r="H119" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="I119" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J119" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K119" s="3" t="s">
         <v>160</v>
@@ -5130,7 +5130,7 @@
     </row>
     <row r="120" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B120" s="4">
         <v>8900</v>
@@ -5151,13 +5151,13 @@
         <v>161</v>
       </c>
       <c r="H120" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I120" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J120" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K120" s="3" t="s">
         <v>162</v>
@@ -5165,7 +5165,7 @@
     </row>
     <row r="121" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B121" s="4">
         <v>1100</v>
@@ -5183,16 +5183,16 @@
         <f>B121/E121</f>
       </c>
       <c r="G121" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H121" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I121" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J121" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K121" s="3" t="s">
         <v>163</v>
@@ -5200,7 +5200,7 @@
     </row>
     <row r="122" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B122" s="4">
         <v>2850</v>
@@ -5221,13 +5221,13 @@
         <v>135</v>
       </c>
       <c r="H122" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I122" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J122" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K122" s="3" t="s">
         <v>164</v>
@@ -5235,7 +5235,7 @@
     </row>
     <row r="123" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B123" s="4">
         <v>2985</v>
@@ -5253,16 +5253,16 @@
         <f>B123/E123</f>
       </c>
       <c r="G123" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H123" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I123" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J123" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K123" s="3" t="s">
         <v>165</v>
@@ -5270,19 +5270,19 @@
     </row>
     <row r="124" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B124" s="4">
-        <v>680</v>
+        <v>1941</v>
       </c>
       <c r="C124" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D124" s="3">
         <v>1</v>
       </c>
       <c r="E124" s="3">
-        <v>22</v>
+        <v>65.1</v>
       </c>
       <c r="F124" s="5">
         <f>B124/E124</f>
@@ -5291,13 +5291,13 @@
         <v>166</v>
       </c>
       <c r="H124" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="I124" s="3" t="s">
-        <v>133</v>
+        <v>13</v>
       </c>
       <c r="J124" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K124" s="3" t="s">
         <v>167</v>
@@ -5305,7 +5305,7 @@
     </row>
     <row r="125" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B125" s="4">
         <v>1200</v>
@@ -5326,13 +5326,13 @@
         <v>142</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I125" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J125" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K125" s="3" t="s">
         <v>168</v>
@@ -5340,7 +5340,7 @@
     </row>
     <row r="126" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B126" s="4">
         <v>1200</v>
@@ -5358,16 +5358,16 @@
         <f>B126/E126</f>
       </c>
       <c r="G126" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I126" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="J126" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K126" s="3" t="s">
         <v>169</v>
@@ -5375,7 +5375,7 @@
     </row>
     <row r="127" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B127" s="4">
         <v>1850</v>
@@ -5393,16 +5393,16 @@
         <f>B127/E127</f>
       </c>
       <c r="G127" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H127" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I127" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="J127" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K127" s="3" t="s">
         <v>170</v>
@@ -5410,7 +5410,7 @@
     </row>
     <row r="128" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B128" s="4">
         <v>1420</v>
@@ -5428,16 +5428,16 @@
         <f>B128/E128</f>
       </c>
       <c r="G128" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I128" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J128" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K128" s="3" t="s">
         <v>171</v>
@@ -5445,7 +5445,7 @@
     </row>
     <row r="129" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B129" s="4">
         <v>1175</v>
@@ -5466,13 +5466,13 @@
         <v>149</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="I129" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="J129" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K129" s="3" t="s">
         <v>172</v>
@@ -5480,7 +5480,7 @@
     </row>
     <row r="130" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B130" s="4">
         <v>1255</v>
@@ -5501,13 +5501,13 @@
         <v>142</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I130" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J130" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K130" s="3" t="s">
         <v>173</v>
@@ -5515,7 +5515,7 @@
     </row>
     <row r="131" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B131" s="4">
         <v>4500</v>
@@ -5536,13 +5536,13 @@
         <v>174</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I131" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J131" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="K131" s="3" t="s">
         <v>175</v>
@@ -5550,7 +5550,7 @@
     </row>
     <row r="132" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B132" s="4">
         <v>2095</v>
@@ -5568,16 +5568,16 @@
         <f>B132/E132</f>
       </c>
       <c r="G132" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="I132" s="3" t="s">
-        <v>132</v>
+        <v>13</v>
       </c>
       <c r="J132" s="3" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="K132" s="3" t="s">
         <v>176</v>

</xml_diff>

<commit_message>
Update listings: 2026-07-07 20:36 UTC
</commit_message>
<xml_diff>
--- a/listings.xlsx
+++ b/listings.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="179">
   <si>
     <t>Source</t>
   </si>
@@ -251,6 +251,9 @@
     <t>https://www.barnes-international.com/en/for-rent/france/paris-16eme/ref-APM-2766079.html</t>
   </si>
   <si>
+    <t>https://www.barnes-international.com/en/for-rent/france/paris-2eme/ref-APM-2765566.html</t>
+  </si>
+  <si>
     <t>https://www.barnes-international.com/en/for-rent/france/paris-17eme/ref-APM-7468343.html</t>
   </si>
   <si>
@@ -404,12 +407,6 @@
     <t>https://www.barnes-international.com/en/for-rent/france/paris-7eme/ref-APM-87067410.html</t>
   </si>
   <si>
-    <t>PARIS 11ÈME</t>
-  </si>
-  <si>
-    <t>https://www.barnes-international.com/en/for-rent/france/paris-11eme/ref-APM-86050237.html</t>
-  </si>
-  <si>
     <t>SeLoger</t>
   </si>
   <si>
@@ -425,46 +422,49 @@
     <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273678077.htm</t>
   </si>
   <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273866199.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/violet-commerce/273849353.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/272541147.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273864065.htm</t>
+  </si>
+  <si>
+    <t>Paris 16ème</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/273639859.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273302365.htm</t>
+  </si>
+  <si>
+    <t>1 220 € /mois</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/suresnes-92/carnot-gambetta/262906241.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/273639863.htm</t>
+  </si>
+  <si>
+    <t>Paris 18ème</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273307251.htm</t>
+  </si>
+  <si>
     <t>Paris 6ème</t>
   </si>
   <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-6eme-75/rennes/272330823.htm</t>
   </si>
   <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273866199.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/violet-commerce/273849353.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/272541147.htm</t>
-  </si>
-  <si>
-    <t>Paris 16ème</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273302365.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273864065.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/273639859.htm</t>
-  </si>
-  <si>
-    <t>1 / 15</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/montreuil-93/ruffins-theophile-sueur-montreau-le-morillon/270926483.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/273639863.htm</t>
-  </si>
-  <si>
-    <t>Paris 18ème</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273307251.htm</t>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/274270579.htm</t>
   </si>
   <si>
     <t>Paris 19ème</t>
@@ -473,9 +473,6 @@
     <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273923913.htm</t>
   </si>
   <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/274270579.htm</t>
-  </si>
-  <si>
     <t>Paris 7ème</t>
   </si>
   <si>
@@ -506,49 +503,46 @@
     <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/273639889.htm</t>
   </si>
   <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/cambronne-garibaldi/274316193.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273630989.htm</t>
+  </si>
+  <si>
+    <t>1 080 € /mois</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/vanves-92/centre-ancien/267289923.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/273639857.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/vaugirard-parc-des-expositions/271629933.htm</t>
+  </si>
+  <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-17eme-75/ternes-maillot/273186559.htm</t>
   </si>
   <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/cambronne-garibaldi/274316193.htm</t>
-  </si>
-  <si>
-    <t>1 941 € /mois</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/issy-les-moulineaux-92/273103027.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-75/273630989.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/273639857.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/271456951.htm</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/vaugirard-parc-des-expositions/271629933.htm</t>
-  </si>
-  <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-18eme-75/goutte-d-or-chateau-rouge/274249093.htm</t>
   </si>
   <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/273639893.htm</t>
   </si>
   <si>
-    <t>Paris 9ème</t>
-  </si>
-  <si>
-    <t>https://www.seloger.com/annonces/locations/appartement/paris-9eme-75/trudaine-maubeuge/273938495.htm</t>
-  </si>
-  <si>
     <t>https://www.seloger.com/annonces/locations/appartement/paris-15eme-75/pasteur-montparnasse/273089161.htm</t>
   </si>
   <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/auteuil-nord/198507995.htm</t>
+  </si>
+  <si>
+    <t>https://www.seloger.com/annonces/locations/appartement/paris-16eme-75/muette-nord/259385227.htm</t>
+  </si>
+  <si>
     <t>Prospector — Paris Listings</t>
   </si>
   <si>
-    <t>Generated: 07/07/2026, 14:37:55</t>
+    <t>Generated: 07/07/2026, 20:36:03</t>
   </si>
   <si>
     <t>Barnes: 100 listings</t>
@@ -1849,7 +1843,7 @@
         <v>11</v>
       </c>
       <c r="B26" s="4">
-        <v>2200</v>
+        <v>2000</v>
       </c>
       <c r="C26" s="3">
         <v>1</v>
@@ -2757,31 +2751,31 @@
         <v>11</v>
       </c>
       <c r="B52" s="4">
-        <v>10600</v>
+        <v>11500</v>
       </c>
       <c r="C52" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D52" s="3">
         <v>3</v>
       </c>
       <c r="E52" s="3">
-        <v>214</v>
+        <v>160</v>
       </c>
       <c r="F52" s="5">
         <f>B52/E52</f>
       </c>
       <c r="G52" s="3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K52" s="3" t="s">
         <v>79</v>
@@ -2792,34 +2786,34 @@
         <v>11</v>
       </c>
       <c r="B53" s="4">
-        <v>10450</v>
+        <v>10600</v>
       </c>
       <c r="C53" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D53" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E53" s="3">
-        <v>156</v>
+        <v>214</v>
       </c>
       <c r="F53" s="5">
         <f>B53/E53</f>
       </c>
       <c r="G53" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K53" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="H53" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I53" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J53" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K53" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="54" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -2827,7 +2821,7 @@
         <v>11</v>
       </c>
       <c r="B54" s="4">
-        <v>10000</v>
+        <v>10450</v>
       </c>
       <c r="C54" s="3">
         <v>3</v>
@@ -2836,22 +2830,22 @@
         <v>2</v>
       </c>
       <c r="E54" s="3">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F54" s="5">
         <f>B54/E54</f>
       </c>
       <c r="G54" s="3" t="s">
-        <v>41</v>
+        <v>81</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K54" s="3" t="s">
         <v>82</v>
@@ -2865,19 +2859,19 @@
         <v>10000</v>
       </c>
       <c r="C55" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D55" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E55" s="3">
-        <v>220</v>
+        <v>153</v>
       </c>
       <c r="F55" s="5">
         <f>B55/E55</f>
       </c>
       <c r="G55" s="3" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>13</v>
@@ -2886,7 +2880,7 @@
         <v>14</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K55" s="3" t="s">
         <v>83</v>
@@ -2900,28 +2894,28 @@
         <v>10000</v>
       </c>
       <c r="C56" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D56" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E56" s="3">
-        <v>188</v>
+        <v>220</v>
       </c>
       <c r="F56" s="5">
         <f>B56/E56</f>
       </c>
       <c r="G56" s="3" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K56" s="3" t="s">
         <v>84</v>
@@ -2932,28 +2926,28 @@
         <v>11</v>
       </c>
       <c r="B57" s="4">
-        <v>9900</v>
+        <v>10000</v>
       </c>
       <c r="C57" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D57" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E57" s="3">
-        <v>146</v>
+        <v>188</v>
       </c>
       <c r="F57" s="5">
         <f>B57/E57</f>
       </c>
       <c r="G57" s="3" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H57" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J57" s="3" t="s">
         <v>13</v>
@@ -2967,16 +2961,16 @@
         <v>11</v>
       </c>
       <c r="B58" s="4">
-        <v>9800</v>
+        <v>9900</v>
       </c>
       <c r="C58" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D58" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E58" s="3">
-        <v>241</v>
+        <v>146</v>
       </c>
       <c r="F58" s="5">
         <f>B58/E58</f>
@@ -2991,7 +2985,7 @@
         <v>14</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K58" s="3" t="s">
         <v>86</v>
@@ -3002,7 +2996,7 @@
         <v>11</v>
       </c>
       <c r="B59" s="4">
-        <v>9000</v>
+        <v>9800</v>
       </c>
       <c r="C59" s="3">
         <v>3</v>
@@ -3011,7 +3005,7 @@
         <v>3</v>
       </c>
       <c r="E59" s="3">
-        <v>163</v>
+        <v>241</v>
       </c>
       <c r="F59" s="5">
         <f>B59/E59</f>
@@ -3026,7 +3020,7 @@
         <v>14</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K59" s="3" t="s">
         <v>87</v>
@@ -3037,22 +3031,22 @@
         <v>11</v>
       </c>
       <c r="B60" s="4">
-        <v>8900</v>
+        <v>9000</v>
       </c>
       <c r="C60" s="3">
         <v>3</v>
       </c>
       <c r="D60" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E60" s="3">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="F60" s="5">
         <f>B60/E60</f>
       </c>
       <c r="G60" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H60" s="3" t="s">
         <v>13</v>
@@ -3061,7 +3055,7 @@
         <v>14</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K60" s="3" t="s">
         <v>88</v>
@@ -3072,7 +3066,7 @@
         <v>11</v>
       </c>
       <c r="B61" s="4">
-        <v>8700</v>
+        <v>8900</v>
       </c>
       <c r="C61" s="3">
         <v>3</v>
@@ -3081,7 +3075,7 @@
         <v>2</v>
       </c>
       <c r="E61" s="3">
-        <v>104</v>
+        <v>152</v>
       </c>
       <c r="F61" s="5">
         <f>B61/E61</f>
@@ -3093,10 +3087,10 @@
         <v>13</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K61" s="3" t="s">
         <v>89</v>
@@ -3107,22 +3101,22 @@
         <v>11</v>
       </c>
       <c r="B62" s="4">
-        <v>8500</v>
+        <v>8700</v>
       </c>
       <c r="C62" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D62" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E62" s="3">
-        <v>231</v>
+        <v>104</v>
       </c>
       <c r="F62" s="5">
         <f>B62/E62</f>
       </c>
       <c r="G62" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H62" s="3" t="s">
         <v>13</v>
@@ -3131,7 +3125,7 @@
         <v>13</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K62" s="3" t="s">
         <v>90</v>
@@ -3145,28 +3139,28 @@
         <v>8500</v>
       </c>
       <c r="C63" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D63" s="3">
         <v>3</v>
       </c>
       <c r="E63" s="3">
-        <v>153</v>
+        <v>231</v>
       </c>
       <c r="F63" s="5">
         <f>B63/E63</f>
       </c>
       <c r="G63" s="3" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="H63" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K63" s="3" t="s">
         <v>91</v>
@@ -3177,31 +3171,31 @@
         <v>11</v>
       </c>
       <c r="B64" s="4">
-        <v>8400</v>
+        <v>8500</v>
       </c>
       <c r="C64" s="3">
         <v>3</v>
       </c>
       <c r="D64" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E64" s="3">
-        <v>238</v>
+        <v>153</v>
       </c>
       <c r="F64" s="5">
         <f>B64/E64</f>
       </c>
       <c r="G64" s="3" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="H64" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K64" s="3" t="s">
         <v>92</v>
@@ -3212,16 +3206,16 @@
         <v>11</v>
       </c>
       <c r="B65" s="4">
-        <v>8000</v>
+        <v>8400</v>
       </c>
       <c r="C65" s="3">
         <v>3</v>
       </c>
       <c r="D65" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E65" s="3">
-        <v>193</v>
+        <v>238</v>
       </c>
       <c r="F65" s="5">
         <f>B65/E65</f>
@@ -3230,13 +3224,13 @@
         <v>41</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K65" s="3" t="s">
         <v>93</v>
@@ -3247,16 +3241,16 @@
         <v>11</v>
       </c>
       <c r="B66" s="4">
-        <v>7800</v>
+        <v>8000</v>
       </c>
       <c r="C66" s="3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D66" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E66" s="3">
-        <v>242</v>
+        <v>193</v>
       </c>
       <c r="F66" s="5">
         <f>B66/E66</f>
@@ -3265,7 +3259,7 @@
         <v>41</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I66" s="3" t="s">
         <v>14</v>
@@ -3282,25 +3276,25 @@
         <v>11</v>
       </c>
       <c r="B67" s="4">
-        <v>7400</v>
+        <v>7800</v>
       </c>
       <c r="C67" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D67" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E67" s="3">
-        <v>166</v>
+        <v>242</v>
       </c>
       <c r="F67" s="5">
         <f>B67/E67</f>
       </c>
       <c r="G67" s="3" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I67" s="3" t="s">
         <v>14</v>
@@ -3317,25 +3311,25 @@
         <v>11</v>
       </c>
       <c r="B68" s="4">
-        <v>7000</v>
+        <v>7400</v>
       </c>
       <c r="C68" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D68" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E68" s="3">
-        <v>81</v>
+        <v>166</v>
       </c>
       <c r="F68" s="5">
         <f>B68/E68</f>
       </c>
       <c r="G68" s="3" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I68" s="3" t="s">
         <v>14</v>
@@ -3352,7 +3346,7 @@
         <v>11</v>
       </c>
       <c r="B69" s="4">
-        <v>6950</v>
+        <v>7000</v>
       </c>
       <c r="C69" s="3">
         <v>2</v>
@@ -3361,13 +3355,13 @@
         <v>2</v>
       </c>
       <c r="E69" s="3">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="F69" s="5">
         <f>B69/E69</f>
       </c>
       <c r="G69" s="3" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="H69" s="3" t="s">
         <v>13</v>
@@ -3387,22 +3381,22 @@
         <v>11</v>
       </c>
       <c r="B70" s="4">
-        <v>6765</v>
+        <v>6950</v>
       </c>
       <c r="C70" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D70" s="3">
         <v>2</v>
       </c>
       <c r="E70" s="3">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="F70" s="5">
         <f>B70/E70</f>
       </c>
       <c r="G70" s="3" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="H70" s="3" t="s">
         <v>13</v>
@@ -3422,28 +3416,28 @@
         <v>11</v>
       </c>
       <c r="B71" s="4">
-        <v>6550</v>
+        <v>6765</v>
       </c>
       <c r="C71" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D71" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E71" s="3">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="F71" s="5">
         <f>B71/E71</f>
       </c>
       <c r="G71" s="3" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="H71" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J71" s="3" t="s">
         <v>13</v>
@@ -3457,28 +3451,28 @@
         <v>11</v>
       </c>
       <c r="B72" s="4">
-        <v>6520</v>
+        <v>6550</v>
       </c>
       <c r="C72" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D72" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E72" s="3">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="F72" s="5">
         <f>B72/E72</f>
       </c>
       <c r="G72" s="3" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H72" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J72" s="3" t="s">
         <v>13</v>
@@ -3492,31 +3486,31 @@
         <v>11</v>
       </c>
       <c r="B73" s="4">
-        <v>6500</v>
+        <v>6520</v>
       </c>
       <c r="C73" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D73" s="3">
         <v>2</v>
       </c>
       <c r="E73" s="3">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F73" s="5">
         <f>B73/E73</f>
       </c>
       <c r="G73" s="3" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H73" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K73" s="3" t="s">
         <v>101</v>
@@ -3530,28 +3524,28 @@
         <v>6500</v>
       </c>
       <c r="C74" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D74" s="3">
         <v>2</v>
       </c>
       <c r="E74" s="3">
-        <v>152</v>
+        <v>125</v>
       </c>
       <c r="F74" s="5">
         <f>B74/E74</f>
       </c>
       <c r="G74" s="3" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H74" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J74" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K74" s="3" t="s">
         <v>102</v>
@@ -3565,25 +3559,25 @@
         <v>6500</v>
       </c>
       <c r="C75" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D75" s="3">
         <v>2</v>
       </c>
       <c r="E75" s="3">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="F75" s="5">
         <f>B75/E75</f>
       </c>
       <c r="G75" s="3" t="s">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J75" s="3" t="s">
         <v>13</v>
@@ -3597,28 +3591,28 @@
         <v>11</v>
       </c>
       <c r="B76" s="4">
-        <v>6000</v>
+        <v>6500</v>
       </c>
       <c r="C76" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D76" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E76" s="3">
-        <v>52</v>
+        <v>115</v>
       </c>
       <c r="F76" s="5">
         <f>B76/E76</f>
       </c>
       <c r="G76" s="3" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J76" s="3" t="s">
         <v>13</v>
@@ -3632,30 +3626,34 @@
         <v>11</v>
       </c>
       <c r="B77" s="4">
-        <v>5800</v>
-      </c>
-      <c r="C77" s="3"/>
-      <c r="D77" s="3"/>
+        <v>6000</v>
+      </c>
+      <c r="C77" s="3">
+        <v>1</v>
+      </c>
+      <c r="D77" s="3">
+        <v>1</v>
+      </c>
       <c r="E77" s="3">
-        <v>105</v>
+        <v>52</v>
       </c>
       <c r="F77" s="5">
         <f>B77/E77</f>
       </c>
       <c r="G77" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J77" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K77" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="H77" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J77" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K77" s="3" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="78" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -3663,22 +3661,18 @@
         <v>11</v>
       </c>
       <c r="B78" s="4">
-        <v>5500</v>
-      </c>
-      <c r="C78" s="3">
-        <v>3</v>
-      </c>
-      <c r="D78" s="3">
-        <v>2</v>
-      </c>
+        <v>5800</v>
+      </c>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
       <c r="E78" s="3">
-        <v>129</v>
+        <v>105</v>
       </c>
       <c r="F78" s="5">
         <f>B78/E78</f>
       </c>
       <c r="G78" s="3" t="s">
-        <v>12</v>
+        <v>106</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>13</v>
@@ -3736,19 +3730,19 @@
         <v>5500</v>
       </c>
       <c r="C80" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D80" s="3">
         <v>2</v>
       </c>
       <c r="E80" s="3">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="F80" s="5">
         <f>B80/E80</f>
       </c>
       <c r="G80" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H80" s="3" t="s">
         <v>13</v>
@@ -3771,13 +3765,13 @@
         <v>5500</v>
       </c>
       <c r="C81" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D81" s="3">
         <v>2</v>
       </c>
       <c r="E81" s="3">
-        <v>152</v>
+        <v>105</v>
       </c>
       <c r="F81" s="5">
         <f>B81/E81</f>
@@ -3792,7 +3786,7 @@
         <v>14</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K81" s="3" t="s">
         <v>110</v>
@@ -3803,16 +3797,16 @@
         <v>11</v>
       </c>
       <c r="B82" s="4">
-        <v>5400</v>
+        <v>5500</v>
       </c>
       <c r="C82" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D82" s="3">
         <v>2</v>
       </c>
       <c r="E82" s="3">
-        <v>91</v>
+        <v>152</v>
       </c>
       <c r="F82" s="5">
         <f>B82/E82</f>
@@ -3824,10 +3818,10 @@
         <v>13</v>
       </c>
       <c r="I82" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J82" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K82" s="3" t="s">
         <v>111</v>
@@ -3838,16 +3832,16 @@
         <v>11</v>
       </c>
       <c r="B83" s="4">
-        <v>5200</v>
+        <v>5400</v>
       </c>
       <c r="C83" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D83" s="3">
         <v>2</v>
       </c>
       <c r="E83" s="3">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F83" s="5">
         <f>B83/E83</f>
@@ -3859,7 +3853,7 @@
         <v>13</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J83" s="3" t="s">
         <v>13</v>
@@ -3873,7 +3867,7 @@
         <v>11</v>
       </c>
       <c r="B84" s="4">
-        <v>5150</v>
+        <v>5200</v>
       </c>
       <c r="C84" s="3">
         <v>3</v>
@@ -3882,19 +3876,19 @@
         <v>2</v>
       </c>
       <c r="E84" s="3">
-        <v>137</v>
+        <v>90</v>
       </c>
       <c r="F84" s="5">
         <f>B84/E84</f>
       </c>
       <c r="G84" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="H84" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J84" s="3" t="s">
         <v>13</v>
@@ -3908,7 +3902,7 @@
         <v>11</v>
       </c>
       <c r="B85" s="4">
-        <v>5073</v>
+        <v>5150</v>
       </c>
       <c r="C85" s="3">
         <v>3</v>
@@ -3917,19 +3911,19 @@
         <v>2</v>
       </c>
       <c r="E85" s="3">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F85" s="5">
         <f>B85/E85</f>
       </c>
       <c r="G85" s="3" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="H85" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J85" s="3" t="s">
         <v>13</v>
@@ -3943,25 +3937,25 @@
         <v>11</v>
       </c>
       <c r="B86" s="4">
-        <v>4900</v>
+        <v>5073</v>
       </c>
       <c r="C86" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D86" s="3">
         <v>2</v>
       </c>
       <c r="E86" s="3">
-        <v>84</v>
+        <v>136</v>
       </c>
       <c r="F86" s="5">
         <f>B86/E86</f>
       </c>
       <c r="G86" s="3" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I86" s="3" t="s">
         <v>14</v>
@@ -3978,31 +3972,31 @@
         <v>11</v>
       </c>
       <c r="B87" s="4">
-        <v>4800</v>
+        <v>4900</v>
       </c>
       <c r="C87" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D87" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E87" s="3">
-        <v>127</v>
+        <v>84</v>
       </c>
       <c r="F87" s="5">
         <f>B87/E87</f>
       </c>
       <c r="G87" s="3" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="H87" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I87" s="3" t="s">
         <v>14</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K87" s="3" t="s">
         <v>116</v>
@@ -4019,7 +4013,7 @@
         <v>3</v>
       </c>
       <c r="D88" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E88" s="3">
         <v>127</v>
@@ -4034,7 +4028,7 @@
         <v>13</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J88" s="3" t="s">
         <v>14</v>
@@ -4057,7 +4051,7 @@
         <v>2</v>
       </c>
       <c r="E89" s="3">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="F89" s="5">
         <f>B89/E89</f>
@@ -4072,7 +4066,7 @@
         <v>13</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K89" s="3" t="s">
         <v>118</v>
@@ -4086,13 +4080,13 @@
         <v>4800</v>
       </c>
       <c r="C90" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D90" s="3">
         <v>2</v>
       </c>
       <c r="E90" s="3">
-        <v>117</v>
+        <v>145</v>
       </c>
       <c r="F90" s="5">
         <f>B90/E90</f>
@@ -4104,7 +4098,7 @@
         <v>13</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J90" s="3" t="s">
         <v>13</v>
@@ -4118,28 +4112,28 @@
         <v>11</v>
       </c>
       <c r="B91" s="4">
-        <v>4500</v>
+        <v>4800</v>
       </c>
       <c r="C91" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D91" s="3">
         <v>2</v>
       </c>
       <c r="E91" s="3">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="F91" s="5">
         <f>B91/E91</f>
       </c>
       <c r="G91" s="3" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H91" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J91" s="3" t="s">
         <v>13</v>
@@ -4153,7 +4147,7 @@
         <v>11</v>
       </c>
       <c r="B92" s="4">
-        <v>4400</v>
+        <v>4500</v>
       </c>
       <c r="C92" s="3">
         <v>3</v>
@@ -4162,19 +4156,19 @@
         <v>2</v>
       </c>
       <c r="E92" s="3">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="F92" s="5">
         <f>B92/E92</f>
       </c>
       <c r="G92" s="3" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H92" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J92" s="3" t="s">
         <v>13</v>
@@ -4188,7 +4182,7 @@
         <v>11</v>
       </c>
       <c r="B93" s="4">
-        <v>4200</v>
+        <v>4400</v>
       </c>
       <c r="C93" s="3">
         <v>3</v>
@@ -4197,13 +4191,13 @@
         <v>2</v>
       </c>
       <c r="E93" s="3">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="F93" s="5">
         <f>B93/E93</f>
       </c>
       <c r="G93" s="3" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="H93" s="3" t="s">
         <v>13</v>
@@ -4223,7 +4217,7 @@
         <v>11</v>
       </c>
       <c r="B94" s="4">
-        <v>4053</v>
+        <v>4200</v>
       </c>
       <c r="C94" s="3">
         <v>3</v>
@@ -4232,13 +4226,13 @@
         <v>2</v>
       </c>
       <c r="E94" s="3">
-        <v>140</v>
+        <v>103</v>
       </c>
       <c r="F94" s="5">
         <f>B94/E94</f>
       </c>
       <c r="G94" s="3" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H94" s="3" t="s">
         <v>13</v>
@@ -4247,7 +4241,7 @@
         <v>14</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K94" s="3" t="s">
         <v>123</v>
@@ -4258,31 +4252,31 @@
         <v>11</v>
       </c>
       <c r="B95" s="4">
-        <v>3900</v>
+        <v>4053</v>
       </c>
       <c r="C95" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D95" s="3">
         <v>2</v>
       </c>
       <c r="E95" s="3">
-        <v>96</v>
+        <v>140</v>
       </c>
       <c r="F95" s="5">
         <f>B95/E95</f>
       </c>
       <c r="G95" s="3" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="H95" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K95" s="3" t="s">
         <v>124</v>
@@ -4296,19 +4290,19 @@
         <v>3900</v>
       </c>
       <c r="C96" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E96" s="3">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="F96" s="5">
         <f>B96/E96</f>
       </c>
       <c r="G96" s="3" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H96" s="3" t="s">
         <v>13</v>
@@ -4328,31 +4322,31 @@
         <v>11</v>
       </c>
       <c r="B97" s="4">
-        <v>3850</v>
+        <v>3900</v>
       </c>
       <c r="C97" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D97" s="3">
         <v>1</v>
       </c>
       <c r="E97" s="3">
-        <v>124</v>
+        <v>68</v>
       </c>
       <c r="F97" s="5">
         <f>B97/E97</f>
       </c>
       <c r="G97" s="3" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H97" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J97" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K97" s="3" t="s">
         <v>126</v>
@@ -4363,22 +4357,22 @@
         <v>11</v>
       </c>
       <c r="B98" s="4">
-        <v>3750</v>
+        <v>3850</v>
       </c>
       <c r="C98" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D98" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E98" s="3">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="F98" s="5">
         <f>B98/E98</f>
       </c>
       <c r="G98" s="3" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="H98" s="3" t="s">
         <v>13</v>
@@ -4398,22 +4392,22 @@
         <v>11</v>
       </c>
       <c r="B99" s="4">
-        <v>3500</v>
+        <v>3750</v>
       </c>
       <c r="C99" s="3">
         <v>2</v>
       </c>
       <c r="D99" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E99" s="3">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="F99" s="5">
         <f>B99/E99</f>
       </c>
       <c r="G99" s="3" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="H99" s="3" t="s">
         <v>13</v>
@@ -4422,7 +4416,7 @@
         <v>14</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="K99" s="3" t="s">
         <v>128</v>
@@ -4436,13 +4430,13 @@
         <v>3500</v>
       </c>
       <c r="C100" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D100" s="3">
         <v>1</v>
       </c>
       <c r="E100" s="3">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="F100" s="5">
         <f>B100/E100</f>
@@ -4451,13 +4445,13 @@
         <v>12</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I100" s="3" t="s">
         <v>14</v>
       </c>
       <c r="J100" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K100" s="3" t="s">
         <v>129</v>
@@ -4471,36 +4465,36 @@
         <v>3500</v>
       </c>
       <c r="C101" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D101" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E101" s="3">
-        <v>101</v>
+        <v>64</v>
       </c>
       <c r="F101" s="5">
         <f>B101/E101</f>
       </c>
       <c r="G101" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I101" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J101" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K101" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="H101" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I101" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J101" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K101" s="3" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="102" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B102" s="4">
         <v>2200</v>
@@ -4518,24 +4512,24 @@
         <f>B102/E102</f>
       </c>
       <c r="G102" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I102" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J102" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K102" s="3" t="s">
         <v>133</v>
-      </c>
-      <c r="H102" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I102" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J102" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K102" s="3" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="103" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B103" s="4">
         <v>7900</v>
@@ -4553,42 +4547,42 @@
         <f>B103/E103</f>
       </c>
       <c r="G103" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I103" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J103" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K103" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="H103" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I103" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J103" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K103" s="3" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="104" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B104" s="4">
-        <v>6330</v>
+        <v>4700</v>
       </c>
       <c r="C104" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D104" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E104" s="3">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="F104" s="5">
         <f>B104/E104</f>
       </c>
       <c r="G104" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H104" s="3" t="s">
         <v>13</v>
@@ -4597,33 +4591,33 @@
         <v>13</v>
       </c>
       <c r="J104" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K104" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="105" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B105" s="4">
-        <v>4700</v>
+        <v>2700</v>
       </c>
       <c r="C105" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D105" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E105" s="3">
-        <v>107</v>
+        <v>47</v>
       </c>
       <c r="F105" s="5">
         <f>B105/E105</f>
       </c>
       <c r="G105" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H105" s="3" t="s">
         <v>13</v>
@@ -4635,50 +4629,50 @@
         <v>14</v>
       </c>
       <c r="K105" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="106" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B106" s="4">
-        <v>2700</v>
+        <v>2250</v>
       </c>
       <c r="C106" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D106" s="3">
         <v>1</v>
       </c>
       <c r="E106" s="3">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F106" s="5">
         <f>B106/E106</f>
       </c>
       <c r="G106" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H106" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J106" s="3" t="s">
         <v>14</v>
       </c>
       <c r="K106" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="107" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B107" s="4">
-        <v>2250</v>
+        <v>1890</v>
       </c>
       <c r="C107" s="3">
         <v>2</v>
@@ -4687,48 +4681,48 @@
         <v>1</v>
       </c>
       <c r="E107" s="3">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="F107" s="5">
         <f>B107/E107</f>
       </c>
       <c r="G107" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H107" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J107" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K107" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="108" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B108" s="4">
-        <v>4150</v>
+        <v>1100</v>
       </c>
       <c r="C108" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D108" s="3">
         <v>1</v>
       </c>
       <c r="E108" s="3">
-        <v>109</v>
+        <v>9.4</v>
       </c>
       <c r="F108" s="5">
         <f>B108/E108</f>
       </c>
       <c r="G108" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H108" s="3" t="s">
         <v>13</v>
@@ -4740,30 +4734,30 @@
         <v>13</v>
       </c>
       <c r="K108" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="109" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B109" s="4">
-        <v>1890</v>
+        <v>4150</v>
       </c>
       <c r="C109" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D109" s="3">
         <v>1</v>
       </c>
       <c r="E109" s="3">
-        <v>38</v>
+        <v>109</v>
       </c>
       <c r="F109" s="5">
         <f>B109/E109</f>
       </c>
       <c r="G109" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="H109" s="3" t="s">
         <v>13</v>
@@ -4775,155 +4769,155 @@
         <v>13</v>
       </c>
       <c r="K109" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="110" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B110" s="4">
-        <v>1100</v>
+        <v>1220</v>
       </c>
       <c r="C110" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D110" s="3">
         <v>1</v>
       </c>
       <c r="E110" s="3">
-        <v>9.4</v>
+        <v>37.9</v>
       </c>
       <c r="F110" s="5">
         <f>B110/E110</f>
       </c>
       <c r="G110" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J110" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K110" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="111" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B111" s="4">
-        <v>1525</v>
+        <v>1100</v>
       </c>
       <c r="C111" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D111" s="3">
         <v>1</v>
       </c>
       <c r="E111" s="3">
-        <v>66.1</v>
+        <v>10.7</v>
       </c>
       <c r="F111" s="5">
         <f>B111/E111</f>
       </c>
       <c r="G111" s="3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I111" s="3" t="s">
         <v>13</v>
       </c>
       <c r="J111" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K111" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="112" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B112" s="4">
-        <v>1100</v>
+        <v>2100</v>
       </c>
       <c r="C112" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D112" s="3">
         <v>1</v>
       </c>
       <c r="E112" s="3">
-        <v>10.7</v>
+        <v>57</v>
       </c>
       <c r="F112" s="5">
         <f>B112/E112</f>
       </c>
       <c r="G112" s="3" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I112" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J112" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K112" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="113" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B113" s="4">
-        <v>2100</v>
+        <v>6330</v>
       </c>
       <c r="C113" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D113" s="3">
         <v>1</v>
       </c>
       <c r="E113" s="3">
-        <v>57</v>
+        <v>98</v>
       </c>
       <c r="F113" s="5">
         <f>B113/E113</f>
       </c>
       <c r="G113" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H113" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I113" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J113" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K113" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="H113" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I113" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="J113" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K113" s="3" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="114" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B114" s="4">
-        <v>1603</v>
+        <v>2000</v>
       </c>
       <c r="C114" s="3">
         <v>2</v>
@@ -4932,13 +4926,13 @@
         <v>1</v>
       </c>
       <c r="E114" s="3">
-        <v>48</v>
+        <v>39.6</v>
       </c>
       <c r="F114" s="5">
         <f>B114/E114</f>
       </c>
       <c r="G114" s="3" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>13</v>
@@ -4950,15 +4944,15 @@
         <v>13</v>
       </c>
       <c r="K114" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="115" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B115" s="4">
-        <v>2200</v>
+        <v>1603</v>
       </c>
       <c r="C115" s="3">
         <v>2</v>
@@ -4967,13 +4961,13 @@
         <v>1</v>
       </c>
       <c r="E115" s="3">
-        <v>39.6</v>
+        <v>48</v>
       </c>
       <c r="F115" s="5">
         <f>B115/E115</f>
       </c>
       <c r="G115" s="3" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="H115" s="3" t="s">
         <v>13</v>
@@ -4985,15 +4979,15 @@
         <v>13</v>
       </c>
       <c r="K115" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="116" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B116" s="4">
-        <v>162190</v>
+        <v>162200</v>
       </c>
       <c r="C116" s="3">
         <v>2</v>
@@ -5008,24 +5002,24 @@
         <f>B116/E116</f>
       </c>
       <c r="G116" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H116" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I116" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J116" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K116" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="H116" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I116" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J116" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K116" s="3" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="117" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B117" s="4">
         <v>3650</v>
@@ -5043,7 +5037,7 @@
         <f>B117/E117</f>
       </c>
       <c r="G117" s="3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>13</v>
@@ -5055,12 +5049,12 @@
         <v>14</v>
       </c>
       <c r="K117" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="118" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B118" s="4">
         <v>7250</v>
@@ -5078,24 +5072,24 @@
         <f>B118/E118</f>
       </c>
       <c r="G118" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H118" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I118" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J118" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K118" s="3" t="s">
         <v>157</v>
-      </c>
-      <c r="H118" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I118" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J118" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K118" s="3" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="119" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B119" s="4">
         <v>1500</v>
@@ -5113,24 +5107,24 @@
         <f>B119/E119</f>
       </c>
       <c r="G119" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I119" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J119" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K119" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="H119" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I119" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J119" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K119" s="3" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="120" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B120" s="4">
         <v>8900</v>
@@ -5148,24 +5142,24 @@
         <f>B120/E120</f>
       </c>
       <c r="G120" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I120" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J120" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K120" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="H120" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I120" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J120" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K120" s="3" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="121" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B121" s="4">
         <v>1100</v>
@@ -5183,7 +5177,7 @@
         <f>B121/E121</f>
       </c>
       <c r="G121" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H121" s="3" t="s">
         <v>13</v>
@@ -5195,30 +5189,30 @@
         <v>13</v>
       </c>
       <c r="K121" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="122" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B122" s="4">
-        <v>2850</v>
+        <v>2985</v>
       </c>
       <c r="C122" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D122" s="3">
         <v>1</v>
       </c>
       <c r="E122" s="3">
-        <v>80</v>
+        <v>89.6</v>
       </c>
       <c r="F122" s="5">
         <f>B122/E122</f>
       </c>
       <c r="G122" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="H122" s="3" t="s">
         <v>13</v>
@@ -5230,30 +5224,30 @@
         <v>14</v>
       </c>
       <c r="K122" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="123" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B123" s="4">
-        <v>2985</v>
+        <v>1200</v>
       </c>
       <c r="C123" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D123" s="3">
         <v>1</v>
       </c>
       <c r="E123" s="3">
-        <v>89.6</v>
+        <v>12.3</v>
       </c>
       <c r="F123" s="5">
         <f>B123/E123</f>
       </c>
       <c r="G123" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="H123" s="3" t="s">
         <v>13</v>
@@ -5262,50 +5256,48 @@
         <v>13</v>
       </c>
       <c r="J123" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K123" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="124" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B124" s="4">
-        <v>1941</v>
+        <v>1080</v>
       </c>
       <c r="C124" s="3">
-        <v>3</v>
-      </c>
-      <c r="D124" s="3">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D124" s="3"/>
       <c r="E124" s="3">
-        <v>65.1</v>
+        <v>31</v>
       </c>
       <c r="F124" s="5">
         <f>B124/E124</f>
       </c>
       <c r="G124" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="H124" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I124" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J124" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K124" s="3" t="s">
         <v>166</v>
-      </c>
-      <c r="H124" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I124" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J124" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K124" s="3" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="125" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B125" s="4">
         <v>1200</v>
@@ -5317,33 +5309,33 @@
         <v>1</v>
       </c>
       <c r="E125" s="3">
-        <v>12.3</v>
+        <v>13.6</v>
       </c>
       <c r="F125" s="5">
         <f>B125/E125</f>
       </c>
       <c r="G125" s="3" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="H125" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I125" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J125" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K125" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="126" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B126" s="4">
-        <v>1200</v>
+        <v>1420</v>
       </c>
       <c r="C126" s="3">
         <v>1</v>
@@ -5352,33 +5344,33 @@
         <v>1</v>
       </c>
       <c r="E126" s="3">
-        <v>13.6</v>
+        <v>37</v>
       </c>
       <c r="F126" s="5">
         <f>B126/E126</f>
       </c>
       <c r="G126" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H126" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I126" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J126" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K126" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="127" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B127" s="4">
-        <v>1850</v>
+        <v>2850</v>
       </c>
       <c r="C127" s="3">
         <v>2</v>
@@ -5387,118 +5379,118 @@
         <v>1</v>
       </c>
       <c r="E127" s="3">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="F127" s="5">
         <f>B127/E127</f>
       </c>
       <c r="G127" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H127" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I127" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J127" s="3" t="s">
         <v>14</v>
       </c>
       <c r="K127" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="128" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B128" s="4">
-        <v>1420</v>
+        <v>1175</v>
       </c>
       <c r="C128" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D128" s="3">
         <v>1</v>
       </c>
       <c r="E128" s="3">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F128" s="5">
         <f>B128/E128</f>
       </c>
       <c r="G128" s="3" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I128" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J128" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K128" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="129" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B129" s="4">
-        <v>1175</v>
+        <v>1255</v>
       </c>
       <c r="C129" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D129" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E129" s="3">
-        <v>33</v>
+        <v>15.3</v>
       </c>
       <c r="F129" s="5">
         <f>B129/E129</f>
       </c>
       <c r="G129" s="3" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I129" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J129" s="3" t="s">
         <v>13</v>
       </c>
       <c r="K129" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="130" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B130" s="4">
-        <v>1255</v>
+        <v>2095</v>
       </c>
       <c r="C130" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D130" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E130" s="3">
-        <v>15.3</v>
+        <v>55</v>
       </c>
       <c r="F130" s="5">
         <f>B130/E130</f>
       </c>
       <c r="G130" s="3" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="H130" s="3" t="s">
         <v>13</v>
@@ -5507,33 +5499,33 @@
         <v>13</v>
       </c>
       <c r="J130" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K130" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="131" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B131" s="4">
-        <v>4500</v>
+        <v>2705</v>
       </c>
       <c r="C131" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D131" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E131" s="3">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="F131" s="5">
         <f>B131/E131</f>
       </c>
       <c r="G131" s="3" t="s">
-        <v>174</v>
+        <v>140</v>
       </c>
       <c r="H131" s="3" t="s">
         <v>13</v>
@@ -5545,15 +5537,15 @@
         <v>13</v>
       </c>
       <c r="K131" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="132" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B132" s="4">
-        <v>2095</v>
+        <v>2985</v>
       </c>
       <c r="C132" s="3">
         <v>2</v>
@@ -5562,25 +5554,25 @@
         <v>1</v>
       </c>
       <c r="E132" s="3">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F132" s="5">
         <f>B132/E132</f>
       </c>
       <c r="G132" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="H132" s="3" t="s">
         <v>13</v>
       </c>
       <c r="I132" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J132" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K132" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -5600,22 +5592,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>